<commit_message>
fix lỗi không thấy tag sau deploy ver 10 FIX ngày hiệu lực
</commit_message>
<xml_diff>
--- a/cung_cap_dl/dieu_xe/xe_sl/sl_mau.xlsx
+++ b/cung_cap_dl/dieu_xe/xe_sl/sl_mau.xlsx
@@ -5,27 +5,37 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Software\rubber-erp\cung_cap_dl\xe_sl\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Software\rubber-erp\cung_cap_dl\dieu_xe\xe_sl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04CA11D7-A535-4787-AAFC-09B3DE752C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2BC1B7-8DFD-47C3-8BDD-376168F2CBE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="20">
   <si>
     <t>Ngày</t>
   </si>
@@ -67,17 +77,35 @@
     <t>2A</t>
   </si>
   <si>
-    <t>22A</t>
+    <t>16A</t>
   </si>
   <si>
-    <t>3A</t>
+    <t>10A</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>11A</t>
+  </si>
+  <si>
+    <t>18A</t>
+  </si>
+  <si>
+    <t>1A</t>
+  </si>
+  <si>
+    <t>19A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -115,8 +143,27 @@
       <family val="2"/>
       <charset val="163"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFF0000"/>
+      <name val="Times New Roman"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -126,6 +173,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -214,10 +273,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -266,8 +326,27 @@
     <xf numFmtId="4" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -546,14 +625,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S74"/>
+  <dimension ref="A1:AA74"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="7" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" s="7" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -592,7 +671,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:19" s="7" customFormat="1" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" s="7" customFormat="1" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5"/>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -643,15 +722,15 @@
       </c>
       <c r="S2" s="5"/>
     </row>
-    <row r="3" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
-        <v>46161</v>
+        <v>46168</v>
       </c>
       <c r="B3" s="9">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
@@ -660,37 +739,45 @@
       <c r="H3" s="10"/>
       <c r="I3" s="10"/>
       <c r="J3" s="11">
-        <v>1850</v>
+        <v>3960</v>
       </c>
       <c r="K3" s="12">
-        <v>54.52</v>
+        <v>55.45</v>
       </c>
       <c r="L3" s="13">
-        <v>1008.62</v>
+        <v>2195.8200000000002</v>
       </c>
       <c r="M3" s="10"/>
       <c r="N3" s="10"/>
       <c r="O3" s="10"/>
       <c r="P3" s="12">
-        <v>26</v>
+        <v>95</v>
       </c>
       <c r="Q3" s="12">
         <v>65</v>
       </c>
       <c r="R3" s="12">
-        <v>16.899999999999999</v>
+        <v>61.75</v>
       </c>
       <c r="S3" s="1"/>
-    </row>
-    <row r="4" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="T3" s="20"/>
+      <c r="U3" s="20"/>
+      <c r="V3" s="21"/>
+      <c r="W3" s="1"/>
+      <c r="X3" s="22"/>
+      <c r="Y3" s="21"/>
+      <c r="Z3" s="20"/>
+      <c r="AA3" s="1"/>
+    </row>
+    <row r="4" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="14">
-        <v>46161</v>
+        <v>46168</v>
       </c>
       <c r="B4" s="15">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
@@ -699,37 +786,45 @@
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
       <c r="J4" s="17">
-        <v>1930</v>
+        <v>4150</v>
       </c>
       <c r="K4" s="18">
-        <v>55.6</v>
+        <v>55.65</v>
       </c>
       <c r="L4" s="19">
-        <v>1073.08</v>
+        <v>2309.48</v>
       </c>
       <c r="M4" s="16"/>
       <c r="N4" s="16"/>
       <c r="O4" s="16"/>
       <c r="P4" s="18">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="Q4" s="18">
         <v>65</v>
       </c>
       <c r="R4" s="18">
-        <v>18.2</v>
+        <v>16.25</v>
       </c>
       <c r="S4" s="1"/>
-    </row>
-    <row r="5" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="T4" s="20"/>
+      <c r="U4" s="20"/>
+      <c r="V4" s="21"/>
+      <c r="W4" s="1"/>
+      <c r="X4" s="22"/>
+      <c r="Y4" s="21"/>
+      <c r="Z4" s="20"/>
+      <c r="AA4" s="1"/>
+    </row>
+    <row r="5" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14">
-        <v>46161</v>
+        <v>46168</v>
       </c>
       <c r="B5" s="15">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
@@ -738,230 +833,453 @@
       <c r="H5" s="16"/>
       <c r="I5" s="16"/>
       <c r="J5" s="17">
-        <v>1870</v>
+        <v>4030</v>
       </c>
       <c r="K5" s="18">
-        <v>55.19</v>
+        <v>54.87</v>
       </c>
       <c r="L5" s="19">
-        <v>1032.05</v>
+        <v>2211.2600000000002</v>
       </c>
       <c r="M5" s="16"/>
       <c r="N5" s="16"/>
       <c r="O5" s="16"/>
       <c r="P5" s="18">
-        <v>26</v>
+        <v>85</v>
       </c>
       <c r="Q5" s="18">
         <v>65</v>
       </c>
       <c r="R5" s="18">
-        <v>16.899999999999999</v>
+        <v>55.25</v>
       </c>
       <c r="S5" s="1"/>
-    </row>
-    <row r="6" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="14"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
+      <c r="V5" s="21"/>
+      <c r="W5" s="1"/>
+      <c r="X5" s="22"/>
+      <c r="Y5" s="21"/>
+      <c r="Z5" s="20"/>
+      <c r="AA5" s="1"/>
+    </row>
+    <row r="6" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="14">
+        <v>46168</v>
+      </c>
+      <c r="B6" s="15">
+        <v>4</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>13</v>
+      </c>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
       <c r="G6" s="16"/>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
+      <c r="J6" s="17">
+        <v>3550</v>
+      </c>
+      <c r="K6" s="18">
+        <v>55.14</v>
+      </c>
+      <c r="L6" s="19">
+        <v>1957.47</v>
+      </c>
       <c r="M6" s="16"/>
       <c r="N6" s="16"/>
       <c r="O6" s="16"/>
-      <c r="P6" s="18"/>
-      <c r="Q6" s="18"/>
-      <c r="R6" s="18"/>
+      <c r="P6" s="18">
+        <v>37</v>
+      </c>
+      <c r="Q6" s="18">
+        <v>65</v>
+      </c>
+      <c r="R6" s="18">
+        <v>24.05</v>
+      </c>
       <c r="S6" s="1"/>
-    </row>
-    <row r="7" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="14"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
+      <c r="T6" s="20"/>
+      <c r="U6" s="20"/>
+      <c r="V6" s="21"/>
+      <c r="W6" s="1"/>
+      <c r="X6" s="22"/>
+      <c r="Y6" s="21"/>
+      <c r="Z6" s="20"/>
+      <c r="AA6" s="1"/>
+    </row>
+    <row r="7" spans="1:27" s="26" customFormat="1" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A7" s="14">
+        <v>46168</v>
+      </c>
+      <c r="B7" s="15">
+        <v>5</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>17</v>
+      </c>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
       <c r="G7" s="16"/>
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="18"/>
-      <c r="L7" s="18"/>
+      <c r="J7" s="17">
+        <v>3660</v>
+      </c>
+      <c r="K7" s="18">
+        <v>55.26</v>
+      </c>
+      <c r="L7" s="19">
+        <v>2022.52</v>
+      </c>
       <c r="M7" s="16"/>
       <c r="N7" s="16"/>
       <c r="O7" s="16"/>
-      <c r="P7" s="18"/>
-      <c r="Q7" s="18"/>
-      <c r="R7" s="18"/>
-      <c r="S7" s="1"/>
-    </row>
-    <row r="8" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="14"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
+      <c r="P7" s="18">
+        <v>96</v>
+      </c>
+      <c r="Q7" s="18">
+        <v>65</v>
+      </c>
+      <c r="R7" s="18">
+        <v>62.4</v>
+      </c>
+      <c r="S7" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="T7" s="21">
+        <v>3660</v>
+      </c>
+      <c r="U7" s="23"/>
+      <c r="V7" s="24"/>
+      <c r="W7" s="24"/>
+      <c r="X7" s="24"/>
+      <c r="Y7" s="24"/>
+      <c r="Z7" s="25"/>
+      <c r="AA7" s="23"/>
+    </row>
+    <row r="8" spans="1:27" s="26" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="14">
+        <v>46168</v>
+      </c>
+      <c r="B8" s="15">
+        <v>6</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>17</v>
+      </c>
       <c r="D8" s="16"/>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
       <c r="I8" s="16"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
+      <c r="J8" s="17">
+        <v>3140</v>
+      </c>
+      <c r="K8" s="18">
+        <v>55.35</v>
+      </c>
+      <c r="L8" s="19">
+        <v>1737.99</v>
+      </c>
       <c r="M8" s="16"/>
       <c r="N8" s="16"/>
       <c r="O8" s="16"/>
-      <c r="P8" s="18"/>
-      <c r="Q8" s="18"/>
-      <c r="R8" s="18"/>
-      <c r="S8" s="1"/>
-    </row>
-    <row r="9" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="14"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15"/>
+      <c r="P8" s="18">
+        <v>105</v>
+      </c>
+      <c r="Q8" s="18">
+        <v>65</v>
+      </c>
+      <c r="R8" s="18">
+        <v>68.25</v>
+      </c>
+      <c r="S8" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="T8" s="21">
+        <v>3140</v>
+      </c>
+      <c r="U8" s="27"/>
+      <c r="V8" s="27"/>
+      <c r="W8" s="27"/>
+      <c r="X8" s="27"/>
+      <c r="Y8" s="27"/>
+      <c r="Z8" s="27"/>
+    </row>
+    <row r="9" spans="1:27" s="26" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="14">
+        <v>46168</v>
+      </c>
+      <c r="B9" s="15">
+        <v>7</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>12</v>
+      </c>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
       <c r="G9" s="16"/>
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="18"/>
-      <c r="L9" s="18"/>
+      <c r="J9" s="17">
+        <v>2630</v>
+      </c>
+      <c r="K9" s="18">
+        <v>55.49</v>
+      </c>
+      <c r="L9" s="19">
+        <v>1459.39</v>
+      </c>
       <c r="M9" s="16"/>
       <c r="N9" s="16"/>
       <c r="O9" s="16"/>
-      <c r="P9" s="18"/>
-      <c r="Q9" s="18"/>
-      <c r="R9" s="18"/>
-      <c r="S9" s="1"/>
-    </row>
-    <row r="10" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="14"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
+      <c r="P9" s="18">
+        <v>78</v>
+      </c>
+      <c r="Q9" s="18">
+        <v>65</v>
+      </c>
+      <c r="R9" s="18">
+        <v>50.7</v>
+      </c>
+      <c r="S9" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="T9" s="21">
+        <v>2630</v>
+      </c>
+      <c r="U9" s="27"/>
+      <c r="V9" s="27"/>
+      <c r="W9" s="27"/>
+      <c r="X9" s="27"/>
+      <c r="Y9" s="27"/>
+      <c r="Z9" s="27"/>
+    </row>
+    <row r="10" spans="1:27" s="26" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="14">
+        <v>46168</v>
+      </c>
+      <c r="B10" s="15">
+        <v>8</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>12</v>
+      </c>
       <c r="D10" s="16"/>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
       <c r="G10" s="16"/>
       <c r="H10" s="16"/>
       <c r="I10" s="16"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="18"/>
-      <c r="L10" s="18"/>
+      <c r="J10" s="17">
+        <v>2880</v>
+      </c>
+      <c r="K10" s="18">
+        <v>54.63</v>
+      </c>
+      <c r="L10" s="19">
+        <v>1573.34</v>
+      </c>
       <c r="M10" s="16"/>
       <c r="N10" s="16"/>
       <c r="O10" s="16"/>
-      <c r="P10" s="18"/>
-      <c r="Q10" s="18"/>
-      <c r="R10" s="18"/>
-      <c r="S10" s="1"/>
-    </row>
-    <row r="11" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="14"/>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
+      <c r="P10" s="18">
+        <v>115</v>
+      </c>
+      <c r="Q10" s="18">
+        <v>65</v>
+      </c>
+      <c r="R10" s="18">
+        <v>74.75</v>
+      </c>
+      <c r="S10" s="23" t="s">
+        <v>15</v>
+      </c>
+      <c r="T10" s="21">
+        <v>2880</v>
+      </c>
+      <c r="U10" s="27"/>
+      <c r="V10" s="27"/>
+      <c r="W10" s="27"/>
+      <c r="X10" s="27"/>
+      <c r="Y10" s="27"/>
+      <c r="Z10" s="27"/>
+    </row>
+    <row r="11" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="14">
+        <v>46168</v>
+      </c>
+      <c r="B11" s="15">
+        <v>9</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>18</v>
+      </c>
       <c r="D11" s="16"/>
       <c r="E11" s="16"/>
       <c r="F11" s="16"/>
       <c r="G11" s="16"/>
       <c r="H11" s="16"/>
       <c r="I11" s="16"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="18"/>
-      <c r="L11" s="18"/>
+      <c r="J11" s="17">
+        <v>2750</v>
+      </c>
+      <c r="K11" s="18">
+        <v>54.1</v>
+      </c>
+      <c r="L11" s="19">
+        <v>1487.75</v>
+      </c>
       <c r="M11" s="16"/>
       <c r="N11" s="16"/>
       <c r="O11" s="16"/>
-      <c r="P11" s="18"/>
-      <c r="Q11" s="18"/>
-      <c r="R11" s="18"/>
+      <c r="P11" s="18">
+        <v>54</v>
+      </c>
+      <c r="Q11" s="18">
+        <v>65</v>
+      </c>
+      <c r="R11" s="18">
+        <v>35.1</v>
+      </c>
       <c r="S11" s="1"/>
     </row>
-    <row r="12" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="14"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
+    <row r="12" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="14">
+        <v>46168</v>
+      </c>
+      <c r="B12" s="15">
+        <v>10</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>18</v>
+      </c>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
       <c r="G12" s="16"/>
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="18"/>
+      <c r="J12" s="17">
+        <v>3140</v>
+      </c>
+      <c r="K12" s="18">
+        <v>55.19</v>
+      </c>
+      <c r="L12" s="19">
+        <v>1732.97</v>
+      </c>
       <c r="M12" s="16"/>
       <c r="N12" s="16"/>
       <c r="O12" s="16"/>
-      <c r="P12" s="18"/>
-      <c r="Q12" s="18"/>
-      <c r="R12" s="18"/>
+      <c r="P12" s="18">
+        <v>46</v>
+      </c>
+      <c r="Q12" s="18">
+        <v>65</v>
+      </c>
+      <c r="R12" s="18">
+        <v>29.9</v>
+      </c>
       <c r="S12" s="1"/>
     </row>
-    <row r="13" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="14"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
+    <row r="13" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="14">
+        <v>46168</v>
+      </c>
+      <c r="B13" s="15">
+        <v>11</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>19</v>
+      </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
       <c r="F13" s="16"/>
       <c r="G13" s="16"/>
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="19"/>
+      <c r="J13" s="17">
+        <v>2910</v>
+      </c>
+      <c r="K13" s="18">
+        <v>55.84</v>
+      </c>
+      <c r="L13" s="19">
+        <v>1624.94</v>
+      </c>
       <c r="M13" s="16"/>
       <c r="N13" s="16"/>
       <c r="O13" s="16"/>
-      <c r="P13" s="18"/>
-      <c r="Q13" s="18"/>
-      <c r="R13" s="18"/>
+      <c r="P13" s="18">
+        <v>17</v>
+      </c>
+      <c r="Q13" s="18">
+        <v>65</v>
+      </c>
+      <c r="R13" s="18">
+        <v>11.05</v>
+      </c>
       <c r="S13" s="1"/>
     </row>
-    <row r="14" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="14"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15"/>
+    <row r="14" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="14">
+        <v>46168</v>
+      </c>
+      <c r="B14" s="15">
+        <v>12</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>19</v>
+      </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
       <c r="F14" s="16"/>
       <c r="G14" s="16"/>
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="19"/>
+      <c r="J14" s="17">
+        <v>3510</v>
+      </c>
+      <c r="K14" s="18">
+        <v>54.82</v>
+      </c>
+      <c r="L14" s="19">
+        <v>1924.18</v>
+      </c>
       <c r="M14" s="16"/>
       <c r="N14" s="16"/>
       <c r="O14" s="16"/>
-      <c r="P14" s="18"/>
-      <c r="Q14" s="18"/>
-      <c r="R14" s="18"/>
+      <c r="P14" s="18">
+        <v>59</v>
+      </c>
+      <c r="Q14" s="18">
+        <v>65</v>
+      </c>
+      <c r="R14" s="18">
+        <v>38.35</v>
+      </c>
       <c r="S14" s="1"/>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
+    <row r="15" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="14"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
+      <c r="C15" s="20"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
       <c r="I15" s="1"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="4"/>
+      <c r="J15" s="21"/>
+      <c r="K15" s="18"/>
+      <c r="L15" s="19"/>
       <c r="M15" s="1"/>
       <c r="N15" s="1"/>
       <c r="O15" s="1"/>
@@ -970,19 +1288,19 @@
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
+    <row r="16" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="14"/>
       <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
+      <c r="C16" s="20"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="4"/>
+      <c r="J16" s="21"/>
+      <c r="K16" s="18"/>
+      <c r="L16" s="19"/>
       <c r="M16" s="1"/>
       <c r="N16" s="1"/>
       <c r="O16" s="1"/>
@@ -991,19 +1309,19 @@
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
+    <row r="17" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="14"/>
       <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+      <c r="C17" s="20"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="4"/>
+      <c r="J17" s="21"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="19"/>
       <c r="M17" s="1"/>
       <c r="N17" s="1"/>
       <c r="O17" s="1"/>
@@ -1012,19 +1330,19 @@
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A18" s="2"/>
+    <row r="18" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="14"/>
       <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
+      <c r="C18" s="20"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="4"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="18"/>
+      <c r="L18" s="19"/>
       <c r="M18" s="1"/>
       <c r="N18" s="1"/>
       <c r="O18" s="1"/>
@@ -1036,7 +1354,6 @@
     <row r="19" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>

</xml_diff>

<commit_message>
fix ngày hiệu lực chỉ điền khi phê duyệt, thêm ghi chú vào lọc sản lượng
</commit_message>
<xml_diff>
--- a/cung_cap_dl/dieu_xe/xe_sl/sl_mau.xlsx
+++ b/cung_cap_dl/dieu_xe/xe_sl/sl_mau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Software\rubber-erp\cung_cap_dl\dieu_xe\xe_sl\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F2BC1B7-8DFD-47C3-8BDD-376168F2CBE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA7A60EC-5E2B-4E83-B3C7-31DF090845B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="19">
   <si>
     <t>Ngày</t>
   </si>
@@ -74,13 +74,7 @@
     <t>Ghi chú</t>
   </si>
   <si>
-    <t>2A</t>
-  </si>
-  <si>
     <t>16A</t>
-  </si>
-  <si>
-    <t>10A</t>
   </si>
   <si>
     <t>T</t>
@@ -89,13 +83,16 @@
     <t>11A</t>
   </si>
   <si>
-    <t>18A</t>
+    <t>22A</t>
   </si>
   <si>
-    <t>1A</t>
+    <t>8A</t>
   </si>
   <si>
-    <t>19A</t>
+    <t>14A</t>
+  </si>
+  <si>
+    <t>5A</t>
   </si>
 </sst>
 </file>
@@ -105,7 +102,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -161,6 +158,14 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="163"/>
     </font>
   </fonts>
   <fills count="5">
@@ -277,7 +282,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -344,6 +349,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -724,13 +735,13 @@
     </row>
     <row r="3" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B3" s="9">
         <v>1</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
@@ -739,25 +750,25 @@
       <c r="H3" s="10"/>
       <c r="I3" s="10"/>
       <c r="J3" s="11">
-        <v>3960</v>
+        <v>4370</v>
       </c>
       <c r="K3" s="12">
-        <v>55.45</v>
+        <v>55.38</v>
       </c>
       <c r="L3" s="13">
-        <v>2195.8200000000002</v>
+        <v>2420.11</v>
       </c>
       <c r="M3" s="10"/>
       <c r="N3" s="10"/>
       <c r="O3" s="10"/>
       <c r="P3" s="12">
-        <v>95</v>
-      </c>
-      <c r="Q3" s="12">
+        <v>39</v>
+      </c>
+      <c r="Q3" s="29">
         <v>65</v>
       </c>
-      <c r="R3" s="12">
-        <v>61.75</v>
+      <c r="R3" s="29">
+        <v>25.35</v>
       </c>
       <c r="S3" s="1"/>
       <c r="T3" s="20"/>
@@ -771,13 +782,13 @@
     </row>
     <row r="4" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="14">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B4" s="15">
         <v>2</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D4" s="16"/>
       <c r="E4" s="16"/>
@@ -786,25 +797,25 @@
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
       <c r="J4" s="17">
-        <v>4150</v>
+        <v>4350</v>
       </c>
       <c r="K4" s="18">
-        <v>55.65</v>
+        <v>55.62</v>
       </c>
       <c r="L4" s="19">
-        <v>2309.48</v>
+        <v>2419.4699999999998</v>
       </c>
       <c r="M4" s="16"/>
       <c r="N4" s="16"/>
       <c r="O4" s="16"/>
       <c r="P4" s="18">
-        <v>25</v>
-      </c>
-      <c r="Q4" s="18">
+        <v>43</v>
+      </c>
+      <c r="Q4" s="28">
         <v>65</v>
       </c>
-      <c r="R4" s="18">
-        <v>16.25</v>
+      <c r="R4" s="28">
+        <v>27.95</v>
       </c>
       <c r="S4" s="1"/>
       <c r="T4" s="20"/>
@@ -818,13 +829,13 @@
     </row>
     <row r="5" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="14">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B5" s="15">
         <v>3</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D5" s="16"/>
       <c r="E5" s="16"/>
@@ -833,25 +844,25 @@
       <c r="H5" s="16"/>
       <c r="I5" s="16"/>
       <c r="J5" s="17">
-        <v>4030</v>
+        <v>5670</v>
       </c>
       <c r="K5" s="18">
-        <v>54.87</v>
+        <v>55.19</v>
       </c>
       <c r="L5" s="19">
-        <v>2211.2600000000002</v>
+        <v>3129.27</v>
       </c>
       <c r="M5" s="16"/>
       <c r="N5" s="16"/>
       <c r="O5" s="16"/>
       <c r="P5" s="18">
-        <v>85</v>
-      </c>
-      <c r="Q5" s="18">
+        <v>61</v>
+      </c>
+      <c r="Q5" s="28">
         <v>65</v>
       </c>
-      <c r="R5" s="18">
-        <v>55.25</v>
+      <c r="R5" s="28">
+        <v>39.65</v>
       </c>
       <c r="S5" s="1"/>
       <c r="T5" s="20"/>
@@ -865,13 +876,13 @@
     </row>
     <row r="6" spans="1:27" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="14">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B6" s="15">
         <v>4</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
@@ -880,25 +891,25 @@
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
       <c r="J6" s="17">
-        <v>3550</v>
+        <v>3720</v>
       </c>
       <c r="K6" s="18">
-        <v>55.14</v>
+        <v>55.34</v>
       </c>
       <c r="L6" s="19">
-        <v>1957.47</v>
+        <v>2058.65</v>
       </c>
       <c r="M6" s="16"/>
       <c r="N6" s="16"/>
       <c r="O6" s="16"/>
       <c r="P6" s="18">
-        <v>37</v>
-      </c>
-      <c r="Q6" s="18">
+        <v>29</v>
+      </c>
+      <c r="Q6" s="28">
         <v>65</v>
       </c>
-      <c r="R6" s="18">
-        <v>24.05</v>
+      <c r="R6" s="28">
+        <v>18.850000000000001</v>
       </c>
       <c r="S6" s="1"/>
       <c r="T6" s="20"/>
@@ -912,7 +923,7 @@
     </row>
     <row r="7" spans="1:27" s="26" customFormat="1" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="14">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B7" s="15">
         <v>5</v>
@@ -927,32 +938,27 @@
       <c r="H7" s="16"/>
       <c r="I7" s="16"/>
       <c r="J7" s="17">
-        <v>3660</v>
+        <v>4120</v>
       </c>
       <c r="K7" s="18">
-        <v>55.26</v>
+        <v>55.66</v>
       </c>
       <c r="L7" s="19">
-        <v>2022.52</v>
+        <v>2293.19</v>
       </c>
       <c r="M7" s="16"/>
       <c r="N7" s="16"/>
       <c r="O7" s="16"/>
       <c r="P7" s="18">
-        <v>96</v>
-      </c>
-      <c r="Q7" s="18">
+        <v>45</v>
+      </c>
+      <c r="Q7" s="28">
         <v>65</v>
       </c>
-      <c r="R7" s="18">
-        <v>62.4</v>
-      </c>
-      <c r="S7" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="T7" s="21">
-        <v>3660</v>
-      </c>
+      <c r="R7" s="28">
+        <v>29.25</v>
+      </c>
+      <c r="T7" s="21"/>
       <c r="U7" s="23"/>
       <c r="V7" s="24"/>
       <c r="W7" s="24"/>
@@ -963,7 +969,7 @@
     </row>
     <row r="8" spans="1:27" s="26" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="14">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B8" s="15">
         <v>6</v>
@@ -978,32 +984,27 @@
       <c r="H8" s="16"/>
       <c r="I8" s="16"/>
       <c r="J8" s="17">
-        <v>3140</v>
+        <v>3910</v>
       </c>
       <c r="K8" s="18">
-        <v>55.35</v>
+        <v>54.96</v>
       </c>
       <c r="L8" s="19">
-        <v>1737.99</v>
+        <v>2148.94</v>
       </c>
       <c r="M8" s="16"/>
       <c r="N8" s="16"/>
       <c r="O8" s="16"/>
       <c r="P8" s="18">
-        <v>105</v>
-      </c>
-      <c r="Q8" s="18">
+        <v>51</v>
+      </c>
+      <c r="Q8" s="28">
         <v>65</v>
       </c>
-      <c r="R8" s="18">
-        <v>68.25</v>
-      </c>
-      <c r="S8" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="T8" s="21">
-        <v>3140</v>
-      </c>
+      <c r="R8" s="28">
+        <v>33.15</v>
+      </c>
+      <c r="T8" s="21"/>
       <c r="U8" s="27"/>
       <c r="V8" s="27"/>
       <c r="W8" s="27"/>
@@ -1013,7 +1014,7 @@
     </row>
     <row r="9" spans="1:27" s="26" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="14">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B9" s="15">
         <v>7</v>
@@ -1028,32 +1029,27 @@
       <c r="H9" s="16"/>
       <c r="I9" s="16"/>
       <c r="J9" s="17">
-        <v>2630</v>
+        <v>2850</v>
       </c>
       <c r="K9" s="18">
-        <v>55.49</v>
+        <v>55.07</v>
       </c>
       <c r="L9" s="19">
-        <v>1459.39</v>
+        <v>1569.5</v>
       </c>
       <c r="M9" s="16"/>
       <c r="N9" s="16"/>
       <c r="O9" s="16"/>
       <c r="P9" s="18">
-        <v>78</v>
-      </c>
-      <c r="Q9" s="18">
+        <v>38</v>
+      </c>
+      <c r="Q9" s="28">
         <v>65</v>
       </c>
-      <c r="R9" s="18">
-        <v>50.7</v>
-      </c>
-      <c r="S9" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="T9" s="21">
-        <v>2630</v>
-      </c>
+      <c r="R9" s="28">
+        <v>24.7</v>
+      </c>
+      <c r="T9" s="21"/>
       <c r="U9" s="27"/>
       <c r="V9" s="27"/>
       <c r="W9" s="27"/>
@@ -1063,7 +1059,7 @@
     </row>
     <row r="10" spans="1:27" s="26" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="14">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B10" s="15">
         <v>8</v>
@@ -1078,32 +1074,27 @@
       <c r="H10" s="16"/>
       <c r="I10" s="16"/>
       <c r="J10" s="17">
-        <v>2880</v>
+        <v>2630</v>
       </c>
       <c r="K10" s="18">
-        <v>54.63</v>
+        <v>54.76</v>
       </c>
       <c r="L10" s="19">
-        <v>1573.34</v>
+        <v>1440.19</v>
       </c>
       <c r="M10" s="16"/>
       <c r="N10" s="16"/>
       <c r="O10" s="16"/>
       <c r="P10" s="18">
-        <v>115</v>
-      </c>
-      <c r="Q10" s="18">
+        <v>37</v>
+      </c>
+      <c r="Q10" s="28">
         <v>65</v>
       </c>
-      <c r="R10" s="18">
-        <v>74.75</v>
-      </c>
-      <c r="S10" s="23" t="s">
-        <v>15</v>
-      </c>
-      <c r="T10" s="21">
-        <v>2880</v>
-      </c>
+      <c r="R10" s="28">
+        <v>24.05</v>
+      </c>
+      <c r="T10" s="21"/>
       <c r="U10" s="27"/>
       <c r="V10" s="27"/>
       <c r="W10" s="27"/>
@@ -1113,7 +1104,7 @@
     </row>
     <row r="11" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="14">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B11" s="15">
         <v>9</v>
@@ -1128,31 +1119,33 @@
       <c r="H11" s="16"/>
       <c r="I11" s="16"/>
       <c r="J11" s="17">
-        <v>2750</v>
+        <v>2490</v>
       </c>
       <c r="K11" s="18">
-        <v>54.1</v>
+        <v>55.54</v>
       </c>
       <c r="L11" s="19">
-        <v>1487.75</v>
+        <v>1382.95</v>
       </c>
       <c r="M11" s="16"/>
       <c r="N11" s="16"/>
       <c r="O11" s="16"/>
       <c r="P11" s="18">
-        <v>54</v>
-      </c>
-      <c r="Q11" s="18">
+        <v>49</v>
+      </c>
+      <c r="Q11" s="28">
         <v>65</v>
       </c>
-      <c r="R11" s="18">
-        <v>35.1</v>
-      </c>
-      <c r="S11" s="1"/>
+      <c r="R11" s="28">
+        <v>31.85</v>
+      </c>
+      <c r="S11" s="23" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="12" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="14">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B12" s="15">
         <v>10</v>
@@ -1167,37 +1160,39 @@
       <c r="H12" s="16"/>
       <c r="I12" s="16"/>
       <c r="J12" s="17">
-        <v>3140</v>
+        <v>3310</v>
       </c>
       <c r="K12" s="18">
-        <v>55.19</v>
+        <v>54.68</v>
       </c>
       <c r="L12" s="19">
-        <v>1732.97</v>
+        <v>1809.91</v>
       </c>
       <c r="M12" s="16"/>
       <c r="N12" s="16"/>
       <c r="O12" s="16"/>
       <c r="P12" s="18">
-        <v>46</v>
-      </c>
-      <c r="Q12" s="18">
+        <v>36</v>
+      </c>
+      <c r="Q12" s="28">
         <v>65</v>
       </c>
-      <c r="R12" s="18">
-        <v>29.9</v>
-      </c>
-      <c r="S12" s="1"/>
+      <c r="R12" s="28">
+        <v>23.4</v>
+      </c>
+      <c r="S12" s="23" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="13" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="14">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B13" s="15">
         <v>11</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
@@ -1206,37 +1201,39 @@
       <c r="H13" s="16"/>
       <c r="I13" s="16"/>
       <c r="J13" s="17">
-        <v>2910</v>
+        <v>3540</v>
       </c>
       <c r="K13" s="18">
-        <v>55.84</v>
+        <v>55.58</v>
       </c>
       <c r="L13" s="19">
-        <v>1624.94</v>
+        <v>1967.53</v>
       </c>
       <c r="M13" s="16"/>
       <c r="N13" s="16"/>
       <c r="O13" s="16"/>
       <c r="P13" s="18">
-        <v>17</v>
-      </c>
-      <c r="Q13" s="18">
+        <v>52</v>
+      </c>
+      <c r="Q13" s="28">
         <v>65</v>
       </c>
-      <c r="R13" s="18">
-        <v>11.05</v>
-      </c>
-      <c r="S13" s="1"/>
+      <c r="R13" s="28">
+        <v>33.799999999999997</v>
+      </c>
+      <c r="S13" s="23" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="14" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="14">
-        <v>46168</v>
+        <v>46173</v>
       </c>
       <c r="B14" s="15">
         <v>12</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
@@ -1245,110 +1242,100 @@
       <c r="H14" s="16"/>
       <c r="I14" s="16"/>
       <c r="J14" s="17">
-        <v>3510</v>
+        <v>3960</v>
       </c>
       <c r="K14" s="18">
-        <v>54.82</v>
+        <v>55.09</v>
       </c>
       <c r="L14" s="19">
-        <v>1924.18</v>
+        <v>2181.56</v>
       </c>
       <c r="M14" s="16"/>
       <c r="N14" s="16"/>
       <c r="O14" s="16"/>
       <c r="P14" s="18">
-        <v>59</v>
-      </c>
-      <c r="Q14" s="18">
+        <v>43</v>
+      </c>
+      <c r="Q14" s="28">
         <v>65</v>
       </c>
-      <c r="R14" s="18">
-        <v>38.35</v>
-      </c>
-      <c r="S14" s="1"/>
+      <c r="R14" s="28">
+        <v>27.95</v>
+      </c>
+      <c r="S14" s="23" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="15" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="21"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="17"/>
       <c r="K15" s="18"/>
       <c r="L15" s="19"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="1"/>
-      <c r="R15" s="1"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="16"/>
       <c r="S15" s="1"/>
     </row>
     <row r="16" spans="1:27" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="14"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="21"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="17"/>
       <c r="K16" s="18"/>
       <c r="L16" s="19"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
-      <c r="Q16" s="1"/>
-      <c r="R16" s="1"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
       <c r="S16" s="1"/>
     </row>
     <row r="17" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="14"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="21"/>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="17"/>
       <c r="K17" s="18"/>
       <c r="L17" s="19"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-      <c r="Q17" s="1"/>
-      <c r="R17" s="1"/>
+      <c r="M17" s="16"/>
+      <c r="N17" s="16"/>
+      <c r="O17" s="16"/>
       <c r="S17" s="1"/>
     </row>
     <row r="18" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="21"/>
+      <c r="B18" s="15"/>
+      <c r="C18" s="15"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="17"/>
       <c r="K18" s="18"/>
       <c r="L18" s="19"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
-      <c r="Q18" s="1"/>
-      <c r="R18" s="1"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
       <c r="S18" s="1"/>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.3">

</xml_diff>